<commit_message>
modified sub-RQ1 result analysis file
</commit_message>
<xml_diff>
--- a/sub-RQ1_result/analysis/result_analysis_excel.xlsx
+++ b/sub-RQ1_result/analysis/result_analysis_excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Master_Winfo\MA_Supply_chain_security\MS_test_system\sub-RQ1_result\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{352EBEDA-C432-4507-BD2F-8EE2C97921FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD5B371-4D52-4476-BF86-4EC3A6F00134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{482212B2-0356-4914-B53B-8802B28615EB}"/>
   </bookViews>

</xml_diff>

<commit_message>
found an problem, updated thesis log
</commit_message>
<xml_diff>
--- a/sub-RQ1_result/analysis/result_analysis_excel.xlsx
+++ b/sub-RQ1_result/analysis/result_analysis_excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Master_Winfo\MA_Supply_chain_security\MS_test_system\sub-RQ1_result\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD5B371-4D52-4476-BF86-4EC3A6F00134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D079F33D-E640-4BD6-94A8-5E059DD0321C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{482212B2-0356-4914-B53B-8802B28615EB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{482212B2-0356-4914-B53B-8802B28615EB}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="2" r:id="rId1"/>
@@ -2950,7 +2950,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2966,6 +2966,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -3257,7 +3258,34 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F29230C-F0E4-43EA-8341-3E01AF9D8D83}" name="results" displayName="results" ref="A1:W433" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:W433" xr:uid="{7F29230C-F0E4-43EA-8341-3E01AF9D8D83}"/>
+  <autoFilter ref="A1:W433" xr:uid="{7F29230C-F0E4-43EA-8341-3E01AF9D8D83}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="java"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="B1d"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="5">
+      <filters>
+        <filter val="B2a"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="6">
+      <filters>
+        <filter val="C1b"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="7">
+      <filters>
+        <filter val="malicious_resolved"/>
+        <filter val="resolution_error"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{A65D53B3-AEE8-4BDA-A007-78AF105B23C7}" uniqueName="1" name="cell_id" queryTableFieldId="1" dataDxfId="42"/>
     <tableColumn id="2" xr3:uid="{FAE1C5D0-B844-4E04-8570-5E7392EC0CD8}" uniqueName="2" name="timestamp" queryTableFieldId="2" dataDxfId="41"/>
@@ -3709,7 +3737,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -3786,7 +3814,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -3863,7 +3891,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -3940,7 +3968,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -4021,7 +4049,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -4102,7 +4130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -4179,7 +4207,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -4250,7 +4278,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -4321,7 +4349,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -4398,7 +4426,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>57</v>
       </c>
@@ -4475,7 +4503,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -4552,7 +4580,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>61</v>
       </c>
@@ -4629,7 +4657,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>63</v>
       </c>
@@ -4700,7 +4728,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -4771,7 +4799,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>68</v>
       </c>
@@ -4848,7 +4876,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>72</v>
       </c>
@@ -4925,7 +4953,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>74</v>
       </c>
@@ -5002,7 +5030,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>76</v>
       </c>
@@ -5079,7 +5107,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>78</v>
       </c>
@@ -5150,7 +5178,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>81</v>
       </c>
@@ -5221,7 +5249,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>83</v>
       </c>
@@ -5298,7 +5326,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>85</v>
       </c>
@@ -5375,7 +5403,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>87</v>
       </c>
@@ -5452,7 +5480,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>89</v>
       </c>
@@ -5529,7 +5557,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>91</v>
       </c>
@@ -5606,7 +5634,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>96</v>
       </c>
@@ -5683,7 +5711,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>98</v>
       </c>
@@ -5760,7 +5788,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>102</v>
       </c>
@@ -5837,7 +5865,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>104</v>
       </c>
@@ -5914,7 +5942,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>106</v>
       </c>
@@ -5991,7 +6019,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>108</v>
       </c>
@@ -6062,7 +6090,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>110</v>
       </c>
@@ -6133,7 +6161,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>112</v>
       </c>
@@ -6210,7 +6238,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>114</v>
       </c>
@@ -6287,7 +6315,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>116</v>
       </c>
@@ -6364,7 +6392,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>118</v>
       </c>
@@ -6441,7 +6469,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>120</v>
       </c>
@@ -6512,7 +6540,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>122</v>
       </c>
@@ -6583,7 +6611,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>124</v>
       </c>
@@ -6660,7 +6688,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>126</v>
       </c>
@@ -6737,7 +6765,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>128</v>
       </c>
@@ -6814,7 +6842,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>130</v>
       </c>
@@ -6891,7 +6919,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>132</v>
       </c>
@@ -6962,7 +6990,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>134</v>
       </c>
@@ -7033,7 +7061,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>136</v>
       </c>
@@ -7110,7 +7138,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>138</v>
       </c>
@@ -7187,7 +7215,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>140</v>
       </c>
@@ -7264,7 +7292,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>142</v>
       </c>
@@ -7341,7 +7369,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>144</v>
       </c>
@@ -7412,7 +7440,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>147</v>
       </c>
@@ -7483,7 +7511,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>149</v>
       </c>
@@ -7554,7 +7582,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>151</v>
       </c>
@@ -7625,7 +7653,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>153</v>
       </c>
@@ -7696,7 +7724,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>155</v>
       </c>
@@ -7767,7 +7795,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>157</v>
       </c>
@@ -7838,7 +7866,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>159</v>
       </c>
@@ -7909,7 +7937,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>161</v>
       </c>
@@ -7986,7 +8014,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>163</v>
       </c>
@@ -8063,7 +8091,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>165</v>
       </c>
@@ -8140,7 +8168,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>167</v>
       </c>
@@ -8217,7 +8245,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>169</v>
       </c>
@@ -8288,7 +8316,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>171</v>
       </c>
@@ -8359,7 +8387,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>173</v>
       </c>
@@ -8436,7 +8464,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>175</v>
       </c>
@@ -8513,7 +8541,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>177</v>
       </c>
@@ -8590,7 +8618,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>179</v>
       </c>
@@ -8667,7 +8695,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>181</v>
       </c>
@@ -8738,7 +8766,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>183</v>
       </c>
@@ -8809,7 +8837,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>185</v>
       </c>
@@ -8886,7 +8914,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>187</v>
       </c>
@@ -8963,7 +8991,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>189</v>
       </c>
@@ -9040,7 +9068,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>191</v>
       </c>
@@ -9117,7 +9145,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>193</v>
       </c>
@@ -9188,7 +9216,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>196</v>
       </c>
@@ -9259,7 +9287,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>198</v>
       </c>
@@ -9330,7 +9358,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>200</v>
       </c>
@@ -9401,7 +9429,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>202</v>
       </c>
@@ -9472,7 +9500,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>204</v>
       </c>
@@ -9543,7 +9571,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>206</v>
       </c>
@@ -9614,7 +9642,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>208</v>
       </c>
@@ -9685,7 +9713,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>210</v>
       </c>
@@ -9762,7 +9790,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>212</v>
       </c>
@@ -9839,7 +9867,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>214</v>
       </c>
@@ -9916,7 +9944,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>216</v>
       </c>
@@ -9993,7 +10021,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>218</v>
       </c>
@@ -10064,7 +10092,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>220</v>
       </c>
@@ -10135,7 +10163,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>222</v>
       </c>
@@ -10212,7 +10240,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>224</v>
       </c>
@@ -10289,7 +10317,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>226</v>
       </c>
@@ -10366,7 +10394,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>228</v>
       </c>
@@ -10443,7 +10471,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>230</v>
       </c>
@@ -10520,7 +10548,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>237</v>
       </c>
@@ -10597,7 +10625,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>240</v>
       </c>
@@ -10674,7 +10702,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="95" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>242</v>
       </c>
@@ -10751,7 +10779,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>246</v>
       </c>
@@ -10828,7 +10856,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>248</v>
       </c>
@@ -10905,7 +10933,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>250</v>
       </c>
@@ -10982,7 +11010,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>252</v>
       </c>
@@ -11059,7 +11087,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>254</v>
       </c>
@@ -11136,7 +11164,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>256</v>
       </c>
@@ -11213,7 +11241,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="102" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>258</v>
       </c>
@@ -11290,7 +11318,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="103" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>260</v>
       </c>
@@ -11367,7 +11395,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>262</v>
       </c>
@@ -11444,7 +11472,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>266</v>
       </c>
@@ -11521,7 +11549,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="106" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>268</v>
       </c>
@@ -11598,7 +11626,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="107" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>270</v>
       </c>
@@ -11675,7 +11703,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>272</v>
       </c>
@@ -11752,7 +11780,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>274</v>
       </c>
@@ -11829,7 +11857,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="110" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>276</v>
       </c>
@@ -11906,7 +11934,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="111" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>278</v>
       </c>
@@ -11983,7 +12011,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>280</v>
       </c>
@@ -12060,7 +12088,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>282</v>
       </c>
@@ -12137,7 +12165,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>286</v>
       </c>
@@ -12214,7 +12242,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>288</v>
       </c>
@@ -12291,7 +12319,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>290</v>
       </c>
@@ -12368,7 +12396,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>292</v>
       </c>
@@ -12445,7 +12473,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>294</v>
       </c>
@@ -12522,7 +12550,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>296</v>
       </c>
@@ -12593,7 +12621,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>298</v>
       </c>
@@ -12664,7 +12692,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="121" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>300</v>
       </c>
@@ -12735,7 +12763,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="122" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>302</v>
       </c>
@@ -12812,7 +12840,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>304</v>
       </c>
@@ -12883,7 +12911,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>306</v>
       </c>
@@ -12960,7 +12988,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="125" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>308</v>
       </c>
@@ -13037,7 +13065,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="126" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>310</v>
       </c>
@@ -13108,7 +13136,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="127" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>312</v>
       </c>
@@ -13185,7 +13213,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="128" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>314</v>
       </c>
@@ -13262,7 +13290,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>318</v>
       </c>
@@ -13339,7 +13367,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>320</v>
       </c>
@@ -13416,7 +13444,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>322</v>
       </c>
@@ -13493,7 +13521,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>326</v>
       </c>
@@ -13570,7 +13598,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>328</v>
       </c>
@@ -13647,7 +13675,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>330</v>
       </c>
@@ -13724,7 +13752,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>332</v>
       </c>
@@ -13801,7 +13829,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>334</v>
       </c>
@@ -13878,7 +13906,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>336</v>
       </c>
@@ -13955,7 +13983,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>338</v>
       </c>
@@ -14032,7 +14060,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>340</v>
       </c>
@@ -14109,7 +14137,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>342</v>
       </c>
@@ -14186,7 +14214,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>344</v>
       </c>
@@ -14263,7 +14291,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>346</v>
       </c>
@@ -14340,7 +14368,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>348</v>
       </c>
@@ -14417,7 +14445,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>350</v>
       </c>
@@ -14494,7 +14522,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>352</v>
       </c>
@@ -14571,7 +14599,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>354</v>
       </c>
@@ -14648,7 +14676,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>356</v>
       </c>
@@ -14725,7 +14753,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>358</v>
       </c>
@@ -14802,7 +14830,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>360</v>
       </c>
@@ -14879,7 +14907,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>362</v>
       </c>
@@ -14956,7 +14984,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>364</v>
       </c>
@@ -15033,7 +15061,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>366</v>
       </c>
@@ -15110,7 +15138,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>368</v>
       </c>
@@ -15187,7 +15215,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>370</v>
       </c>
@@ -15264,7 +15292,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>372</v>
       </c>
@@ -15335,7 +15363,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>374</v>
       </c>
@@ -15406,7 +15434,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>376</v>
       </c>
@@ -15477,7 +15505,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>378</v>
       </c>
@@ -15554,7 +15582,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>380</v>
       </c>
@@ -15625,7 +15653,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>382</v>
       </c>
@@ -15702,7 +15730,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>384</v>
       </c>
@@ -15779,7 +15807,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>386</v>
       </c>
@@ -15850,7 +15878,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>388</v>
       </c>
@@ -15927,7 +15955,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>390</v>
       </c>
@@ -15998,7 +16026,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>392</v>
       </c>
@@ -16069,7 +16097,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>394</v>
       </c>
@@ -16140,7 +16168,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>396</v>
       </c>
@@ -16211,7 +16239,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>398</v>
       </c>
@@ -16282,7 +16310,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>400</v>
       </c>
@@ -16353,7 +16381,7 @@
         <v/>
       </c>
     </row>
-    <row r="170" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>402</v>
       </c>
@@ -16424,7 +16452,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>404</v>
       </c>
@@ -16495,7 +16523,7 @@
         <v/>
       </c>
     </row>
-    <row r="172" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>406</v>
       </c>
@@ -16566,7 +16594,7 @@
         <v/>
       </c>
     </row>
-    <row r="173" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>408</v>
       </c>
@@ -16643,7 +16671,7 @@
         <v/>
       </c>
     </row>
-    <row r="174" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>412</v>
       </c>
@@ -16720,7 +16748,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>414</v>
       </c>
@@ -16797,7 +16825,7 @@
         <v/>
       </c>
     </row>
-    <row r="176" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>416</v>
       </c>
@@ -16874,7 +16902,7 @@
         <v/>
       </c>
     </row>
-    <row r="177" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>418</v>
       </c>
@@ -16951,7 +16979,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>420</v>
       </c>
@@ -17028,7 +17056,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>422</v>
       </c>
@@ -17105,7 +17133,7 @@
         <v/>
       </c>
     </row>
-    <row r="180" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>424</v>
       </c>
@@ -17182,7 +17210,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>426</v>
       </c>
@@ -17259,7 +17287,7 @@
         <v/>
       </c>
     </row>
-    <row r="182" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>428</v>
       </c>
@@ -17336,7 +17364,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>430</v>
       </c>
@@ -17413,7 +17441,7 @@
         <v/>
       </c>
     </row>
-    <row r="184" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>432</v>
       </c>
@@ -17490,7 +17518,7 @@
         <v/>
       </c>
     </row>
-    <row r="185" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>434</v>
       </c>
@@ -17567,7 +17595,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>436</v>
       </c>
@@ -17644,7 +17672,7 @@
         <v/>
       </c>
     </row>
-    <row r="187" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>438</v>
       </c>
@@ -17721,7 +17749,7 @@
         <v/>
       </c>
     </row>
-    <row r="188" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>440</v>
       </c>
@@ -17798,7 +17826,7 @@
         <v/>
       </c>
     </row>
-    <row r="189" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>442</v>
       </c>
@@ -17875,7 +17903,7 @@
         <v/>
       </c>
     </row>
-    <row r="190" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>444</v>
       </c>
@@ -17952,7 +17980,7 @@
         <v/>
       </c>
     </row>
-    <row r="191" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>446</v>
       </c>
@@ -18023,7 +18051,7 @@
         <v/>
       </c>
     </row>
-    <row r="192" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>448</v>
       </c>
@@ -18094,7 +18122,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>450</v>
       </c>
@@ -18165,7 +18193,7 @@
         <v/>
       </c>
     </row>
-    <row r="194" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>452</v>
       </c>
@@ -18242,7 +18270,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>454</v>
       </c>
@@ -18313,7 +18341,7 @@
         <v/>
       </c>
     </row>
-    <row r="196" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>456</v>
       </c>
@@ -18390,7 +18418,7 @@
         <v/>
       </c>
     </row>
-    <row r="197" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>458</v>
       </c>
@@ -18467,7 +18495,7 @@
         <v/>
       </c>
     </row>
-    <row r="198" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>460</v>
       </c>
@@ -18538,7 +18566,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>462</v>
       </c>
@@ -18615,7 +18643,7 @@
         <v/>
       </c>
     </row>
-    <row r="200" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>464</v>
       </c>
@@ -18686,7 +18714,7 @@
         <v/>
       </c>
     </row>
-    <row r="201" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>466</v>
       </c>
@@ -18757,7 +18785,7 @@
         <v/>
       </c>
     </row>
-    <row r="202" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>468</v>
       </c>
@@ -18828,7 +18856,7 @@
         <v/>
       </c>
     </row>
-    <row r="203" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>470</v>
       </c>
@@ -18899,7 +18927,7 @@
         <v/>
       </c>
     </row>
-    <row r="204" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>472</v>
       </c>
@@ -18970,7 +18998,7 @@
         <v/>
       </c>
     </row>
-    <row r="205" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>474</v>
       </c>
@@ -19041,7 +19069,7 @@
         <v/>
       </c>
     </row>
-    <row r="206" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>476</v>
       </c>
@@ -19112,7 +19140,7 @@
         <v/>
       </c>
     </row>
-    <row r="207" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>478</v>
       </c>
@@ -19183,7 +19211,7 @@
         <v/>
       </c>
     </row>
-    <row r="208" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>480</v>
       </c>
@@ -19254,7 +19282,7 @@
         <v/>
       </c>
     </row>
-    <row r="209" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>482</v>
       </c>
@@ -19331,7 +19359,7 @@
         <v/>
       </c>
     </row>
-    <row r="210" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>484</v>
       </c>
@@ -19408,7 +19436,7 @@
         <v/>
       </c>
     </row>
-    <row r="211" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>486</v>
       </c>
@@ -19485,7 +19513,7 @@
         <v/>
       </c>
     </row>
-    <row r="212" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>488</v>
       </c>
@@ -19562,7 +19590,7 @@
         <v/>
       </c>
     </row>
-    <row r="213" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>490</v>
       </c>
@@ -19639,7 +19667,7 @@
         <v/>
       </c>
     </row>
-    <row r="214" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>492</v>
       </c>
@@ -19716,7 +19744,7 @@
         <v/>
       </c>
     </row>
-    <row r="215" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>494</v>
       </c>
@@ -19793,7 +19821,7 @@
         <v/>
       </c>
     </row>
-    <row r="216" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>496</v>
       </c>
@@ -19870,7 +19898,7 @@
         <v/>
       </c>
     </row>
-    <row r="217" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>498</v>
       </c>
@@ -19947,7 +19975,7 @@
         <v/>
       </c>
     </row>
-    <row r="218" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>500</v>
       </c>
@@ -20018,7 +20046,7 @@
         <v/>
       </c>
     </row>
-    <row r="219" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>502</v>
       </c>
@@ -20089,7 +20117,7 @@
         <v/>
       </c>
     </row>
-    <row r="220" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>504</v>
       </c>
@@ -20160,7 +20188,7 @@
         <v/>
       </c>
     </row>
-    <row r="221" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>506</v>
       </c>
@@ -20237,7 +20265,7 @@
         <v/>
       </c>
     </row>
-    <row r="222" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>508</v>
       </c>
@@ -20308,7 +20336,7 @@
         <v/>
       </c>
     </row>
-    <row r="223" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>510</v>
       </c>
@@ -20385,7 +20413,7 @@
         <v/>
       </c>
     </row>
-    <row r="224" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>512</v>
       </c>
@@ -20462,7 +20490,7 @@
         <v/>
       </c>
     </row>
-    <row r="225" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>514</v>
       </c>
@@ -20533,7 +20561,7 @@
         <v/>
       </c>
     </row>
-    <row r="226" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>516</v>
       </c>
@@ -20610,7 +20638,7 @@
         <v/>
       </c>
     </row>
-    <row r="227" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>518</v>
       </c>
@@ -20687,7 +20715,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="228" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>525</v>
       </c>
@@ -20764,7 +20792,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="229" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>527</v>
       </c>
@@ -20841,7 +20869,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="230" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>529</v>
       </c>
@@ -20918,7 +20946,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="231" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>533</v>
       </c>
@@ -20995,7 +21023,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="232" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>535</v>
       </c>
@@ -21072,7 +21100,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="233" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>537</v>
       </c>
@@ -21149,7 +21177,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="234" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>539</v>
       </c>
@@ -21226,7 +21254,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="235" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>541</v>
       </c>
@@ -21303,7 +21331,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="236" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>543</v>
       </c>
@@ -21380,7 +21408,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="237" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>547</v>
       </c>
@@ -21457,7 +21485,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="238" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>549</v>
       </c>
@@ -21534,7 +21562,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="239" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>551</v>
       </c>
@@ -21611,7 +21639,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="240" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>553</v>
       </c>
@@ -21688,7 +21716,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="241" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>555</v>
       </c>
@@ -21765,7 +21793,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="242" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>557</v>
       </c>
@@ -21842,7 +21870,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="243" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>561</v>
       </c>
@@ -21919,7 +21947,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="244" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>563</v>
       </c>
@@ -21996,7 +22024,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="245" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>565</v>
       </c>
@@ -22089,7 +22117,7 @@
       <c r="G246" t="s">
         <v>238</v>
       </c>
-      <c r="H246" t="s">
+      <c r="H246" s="13" t="s">
         <v>48</v>
       </c>
       <c r="I246" t="s">
@@ -22144,7 +22172,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="247" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>569</v>
       </c>
@@ -22215,7 +22243,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="248" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>571</v>
       </c>
@@ -22292,7 +22320,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="249" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>573</v>
       </c>
@@ -22369,7 +22397,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="250" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>575</v>
       </c>
@@ -22446,7 +22474,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="251" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>577</v>
       </c>
@@ -22523,7 +22551,7 @@
         <v/>
       </c>
     </row>
-    <row r="252" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>581</v>
       </c>
@@ -22600,7 +22628,7 @@
         <v/>
       </c>
     </row>
-    <row r="253" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>583</v>
       </c>
@@ -22677,7 +22705,7 @@
         <v/>
       </c>
     </row>
-    <row r="254" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>585</v>
       </c>
@@ -22754,7 +22782,7 @@
         <v/>
       </c>
     </row>
-    <row r="255" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>589</v>
       </c>
@@ -22831,7 +22859,7 @@
         <v/>
       </c>
     </row>
-    <row r="256" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>591</v>
       </c>
@@ -22908,7 +22936,7 @@
         <v/>
       </c>
     </row>
-    <row r="257" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>593</v>
       </c>
@@ -22985,7 +23013,7 @@
         <v/>
       </c>
     </row>
-    <row r="258" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>595</v>
       </c>
@@ -23062,7 +23090,7 @@
         <v/>
       </c>
     </row>
-    <row r="259" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>597</v>
       </c>
@@ -23139,7 +23167,7 @@
         <v/>
       </c>
     </row>
-    <row r="260" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>599</v>
       </c>
@@ -23216,7 +23244,7 @@
         <v/>
       </c>
     </row>
-    <row r="261" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>601</v>
       </c>
@@ -23293,7 +23321,7 @@
         <v/>
       </c>
     </row>
-    <row r="262" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>603</v>
       </c>
@@ -23370,7 +23398,7 @@
         <v/>
       </c>
     </row>
-    <row r="263" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>605</v>
       </c>
@@ -23447,7 +23475,7 @@
         <v/>
       </c>
     </row>
-    <row r="264" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>607</v>
       </c>
@@ -23524,7 +23552,7 @@
         <v/>
       </c>
     </row>
-    <row r="265" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>609</v>
       </c>
@@ -23601,7 +23629,7 @@
         <v/>
       </c>
     </row>
-    <row r="266" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>611</v>
       </c>
@@ -23678,7 +23706,7 @@
         <v/>
       </c>
     </row>
-    <row r="267" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>613</v>
       </c>
@@ -23755,7 +23783,7 @@
         <v/>
       </c>
     </row>
-    <row r="268" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>615</v>
       </c>
@@ -23832,7 +23860,7 @@
         <v/>
       </c>
     </row>
-    <row r="269" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>617</v>
       </c>
@@ -23925,7 +23953,7 @@
       <c r="G270" t="s">
         <v>238</v>
       </c>
-      <c r="H270" t="s">
+      <c r="H270" s="13" t="s">
         <v>48</v>
       </c>
       <c r="I270" t="s">
@@ -23980,7 +24008,7 @@
         <v/>
       </c>
     </row>
-    <row r="271" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>621</v>
       </c>
@@ -24051,7 +24079,7 @@
         <v/>
       </c>
     </row>
-    <row r="272" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>623</v>
       </c>
@@ -24128,7 +24156,7 @@
         <v/>
       </c>
     </row>
-    <row r="273" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>625</v>
       </c>
@@ -24205,7 +24233,7 @@
         <v/>
       </c>
     </row>
-    <row r="274" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>627</v>
       </c>
@@ -24282,7 +24310,7 @@
         <v/>
       </c>
     </row>
-    <row r="275" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>629</v>
       </c>
@@ -24353,7 +24381,7 @@
         <v/>
       </c>
     </row>
-    <row r="276" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>631</v>
       </c>
@@ -24430,7 +24458,7 @@
         <v/>
       </c>
     </row>
-    <row r="277" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>635</v>
       </c>
@@ -24501,7 +24529,7 @@
         <v/>
       </c>
     </row>
-    <row r="278" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>637</v>
       </c>
@@ -24572,7 +24600,7 @@
         <v/>
       </c>
     </row>
-    <row r="279" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>639</v>
       </c>
@@ -24649,7 +24677,7 @@
         <v/>
       </c>
     </row>
-    <row r="280" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>643</v>
       </c>
@@ -24720,7 +24748,7 @@
         <v/>
       </c>
     </row>
-    <row r="281" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>645</v>
       </c>
@@ -24797,7 +24825,7 @@
         <v/>
       </c>
     </row>
-    <row r="282" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>647</v>
       </c>
@@ -24874,7 +24902,7 @@
         <v/>
       </c>
     </row>
-    <row r="283" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>649</v>
       </c>
@@ -24951,7 +24979,7 @@
         <v/>
       </c>
     </row>
-    <row r="284" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>651</v>
       </c>
@@ -25028,7 +25056,7 @@
         <v/>
       </c>
     </row>
-    <row r="285" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>653</v>
       </c>
@@ -25105,7 +25133,7 @@
         <v/>
       </c>
     </row>
-    <row r="286" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>655</v>
       </c>
@@ -25182,7 +25210,7 @@
         <v/>
       </c>
     </row>
-    <row r="287" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>657</v>
       </c>
@@ -25259,7 +25287,7 @@
         <v/>
       </c>
     </row>
-    <row r="288" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>659</v>
       </c>
@@ -25336,7 +25364,7 @@
         <v/>
       </c>
     </row>
-    <row r="289" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>661</v>
       </c>
@@ -25413,7 +25441,7 @@
         <v/>
       </c>
     </row>
-    <row r="290" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>663</v>
       </c>
@@ -25490,7 +25518,7 @@
         <v/>
       </c>
     </row>
-    <row r="291" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>665</v>
       </c>
@@ -25567,7 +25595,7 @@
         <v/>
       </c>
     </row>
-    <row r="292" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>667</v>
       </c>
@@ -25644,7 +25672,7 @@
         <v/>
       </c>
     </row>
-    <row r="293" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>669</v>
       </c>
@@ -25737,7 +25765,7 @@
       <c r="G294" t="s">
         <v>238</v>
       </c>
-      <c r="H294" t="s">
+      <c r="H294" s="13" t="s">
         <v>48</v>
       </c>
       <c r="I294" t="s">
@@ -25792,7 +25820,7 @@
         <v/>
       </c>
     </row>
-    <row r="295" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>673</v>
       </c>
@@ -25863,7 +25891,7 @@
         <v/>
       </c>
     </row>
-    <row r="296" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>675</v>
       </c>
@@ -25940,7 +25968,7 @@
         <v/>
       </c>
     </row>
-    <row r="297" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>677</v>
       </c>
@@ -26017,7 +26045,7 @@
         <v/>
       </c>
     </row>
-    <row r="298" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>679</v>
       </c>
@@ -26094,7 +26122,7 @@
         <v/>
       </c>
     </row>
-    <row r="299" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>681</v>
       </c>
@@ -26171,7 +26199,7 @@
         <v/>
       </c>
     </row>
-    <row r="300" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>683</v>
       </c>
@@ -26248,7 +26276,7 @@
         <v/>
       </c>
     </row>
-    <row r="301" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>685</v>
       </c>
@@ -26325,7 +26353,7 @@
         <v/>
       </c>
     </row>
-    <row r="302" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>687</v>
       </c>
@@ -26402,7 +26430,7 @@
         <v/>
       </c>
     </row>
-    <row r="303" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>689</v>
       </c>
@@ -26479,7 +26507,7 @@
         <v/>
       </c>
     </row>
-    <row r="304" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>691</v>
       </c>
@@ -26556,7 +26584,7 @@
         <v/>
       </c>
     </row>
-    <row r="305" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>693</v>
       </c>
@@ -26633,7 +26661,7 @@
         <v/>
       </c>
     </row>
-    <row r="306" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>695</v>
       </c>
@@ -26710,7 +26738,7 @@
         <v/>
       </c>
     </row>
-    <row r="307" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>697</v>
       </c>
@@ -26787,7 +26815,7 @@
         <v/>
       </c>
     </row>
-    <row r="308" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>699</v>
       </c>
@@ -26864,7 +26892,7 @@
         <v/>
       </c>
     </row>
-    <row r="309" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>701</v>
       </c>
@@ -26941,7 +26969,7 @@
         <v/>
       </c>
     </row>
-    <row r="310" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>703</v>
       </c>
@@ -27018,7 +27046,7 @@
         <v/>
       </c>
     </row>
-    <row r="311" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>705</v>
       </c>
@@ -27111,7 +27139,7 @@
       <c r="G312" t="s">
         <v>238</v>
       </c>
-      <c r="H312" t="s">
+      <c r="H312" s="13" t="s">
         <v>48</v>
       </c>
       <c r="I312" t="s">
@@ -27166,7 +27194,7 @@
         <v/>
       </c>
     </row>
-    <row r="313" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>709</v>
       </c>
@@ -27237,7 +27265,7 @@
         <v/>
       </c>
     </row>
-    <row r="314" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>711</v>
       </c>
@@ -27314,7 +27342,7 @@
         <v/>
       </c>
     </row>
-    <row r="315" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>713</v>
       </c>
@@ -27391,7 +27419,7 @@
         <v/>
       </c>
     </row>
-    <row r="316" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>715</v>
       </c>
@@ -27468,7 +27496,7 @@
         <v/>
       </c>
     </row>
-    <row r="317" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>717</v>
       </c>
@@ -27545,7 +27573,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="318" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>722</v>
       </c>
@@ -27622,7 +27650,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="319" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>724</v>
       </c>
@@ -27699,7 +27727,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="320" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>726</v>
       </c>
@@ -27770,7 +27798,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="321" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>728</v>
       </c>
@@ -27847,7 +27875,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="322" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>730</v>
       </c>
@@ -27924,7 +27952,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="323" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>732</v>
       </c>
@@ -27995,7 +28023,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="324" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>734</v>
       </c>
@@ -28072,7 +28100,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="325" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>736</v>
       </c>
@@ -28149,7 +28177,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="326" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>738</v>
       </c>
@@ -28220,7 +28248,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="327" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>740</v>
       </c>
@@ -28297,7 +28325,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="328" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>742</v>
       </c>
@@ -28374,7 +28402,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="329" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>744</v>
       </c>
@@ -28451,7 +28479,7 @@
         <v/>
       </c>
     </row>
-    <row r="330" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>746</v>
       </c>
@@ -28528,7 +28556,7 @@
         <v/>
       </c>
     </row>
-    <row r="331" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>748</v>
       </c>
@@ -28605,7 +28633,7 @@
         <v/>
       </c>
     </row>
-    <row r="332" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>750</v>
       </c>
@@ -28676,7 +28704,7 @@
         <v/>
       </c>
     </row>
-    <row r="333" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>752</v>
       </c>
@@ -28753,7 +28781,7 @@
         <v/>
       </c>
     </row>
-    <row r="334" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>754</v>
       </c>
@@ -28830,7 +28858,7 @@
         <v/>
       </c>
     </row>
-    <row r="335" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>756</v>
       </c>
@@ -28901,7 +28929,7 @@
         <v/>
       </c>
     </row>
-    <row r="336" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>758</v>
       </c>
@@ -28978,7 +29006,7 @@
         <v/>
       </c>
     </row>
-    <row r="337" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>760</v>
       </c>
@@ -29055,7 +29083,7 @@
         <v/>
       </c>
     </row>
-    <row r="338" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>762</v>
       </c>
@@ -29126,7 +29154,7 @@
         <v/>
       </c>
     </row>
-    <row r="339" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>764</v>
       </c>
@@ -29203,7 +29231,7 @@
         <v/>
       </c>
     </row>
-    <row r="340" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>766</v>
       </c>
@@ -29280,7 +29308,7 @@
         <v/>
       </c>
     </row>
-    <row r="341" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>768</v>
       </c>
@@ -29357,7 +29385,7 @@
         <v/>
       </c>
     </row>
-    <row r="342" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>770</v>
       </c>
@@ -29434,7 +29462,7 @@
         <v/>
       </c>
     </row>
-    <row r="343" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>774</v>
       </c>
@@ -29511,7 +29539,7 @@
         <v/>
       </c>
     </row>
-    <row r="344" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>776</v>
       </c>
@@ -29582,7 +29610,7 @@
         <v/>
       </c>
     </row>
-    <row r="345" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>778</v>
       </c>
@@ -29659,7 +29687,7 @@
         <v/>
       </c>
     </row>
-    <row r="346" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>780</v>
       </c>
@@ -29736,7 +29764,7 @@
         <v/>
       </c>
     </row>
-    <row r="347" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>782</v>
       </c>
@@ -29807,7 +29835,7 @@
         <v/>
       </c>
     </row>
-    <row r="348" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>784</v>
       </c>
@@ -29884,7 +29912,7 @@
         <v/>
       </c>
     </row>
-    <row r="349" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>786</v>
       </c>
@@ -29961,7 +29989,7 @@
         <v/>
       </c>
     </row>
-    <row r="350" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>788</v>
       </c>
@@ -30032,7 +30060,7 @@
         <v/>
       </c>
     </row>
-    <row r="351" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>790</v>
       </c>
@@ -30109,7 +30137,7 @@
         <v/>
       </c>
     </row>
-    <row r="352" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>792</v>
       </c>
@@ -30186,7 +30214,7 @@
         <v/>
       </c>
     </row>
-    <row r="353" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>794</v>
       </c>
@@ -30263,7 +30291,7 @@
         <v/>
       </c>
     </row>
-    <row r="354" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>796</v>
       </c>
@@ -30340,7 +30368,7 @@
         <v/>
       </c>
     </row>
-    <row r="355" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>798</v>
       </c>
@@ -30417,7 +30445,7 @@
         <v/>
       </c>
     </row>
-    <row r="356" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>800</v>
       </c>
@@ -30488,7 +30516,7 @@
         <v/>
       </c>
     </row>
-    <row r="357" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>802</v>
       </c>
@@ -30565,7 +30593,7 @@
         <v/>
       </c>
     </row>
-    <row r="358" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>804</v>
       </c>
@@ -30642,7 +30670,7 @@
         <v/>
       </c>
     </row>
-    <row r="359" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>806</v>
       </c>
@@ -30713,7 +30741,7 @@
         <v/>
       </c>
     </row>
-    <row r="360" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>808</v>
       </c>
@@ -30790,7 +30818,7 @@
         <v/>
       </c>
     </row>
-    <row r="361" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>810</v>
       </c>
@@ -30867,7 +30895,7 @@
         <v/>
       </c>
     </row>
-    <row r="362" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>812</v>
       </c>
@@ -30935,7 +30963,7 @@
         <v/>
       </c>
     </row>
-    <row r="363" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>814</v>
       </c>
@@ -31003,7 +31031,7 @@
         <v/>
       </c>
     </row>
-    <row r="364" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>815</v>
       </c>
@@ -31071,7 +31099,7 @@
         <v/>
       </c>
     </row>
-    <row r="365" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>816</v>
       </c>
@@ -31139,7 +31167,7 @@
         <v/>
       </c>
     </row>
-    <row r="366" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>817</v>
       </c>
@@ -31207,7 +31235,7 @@
         <v/>
       </c>
     </row>
-    <row r="367" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>818</v>
       </c>
@@ -31275,7 +31303,7 @@
         <v/>
       </c>
     </row>
-    <row r="368" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>819</v>
       </c>
@@ -31343,7 +31371,7 @@
         <v/>
       </c>
     </row>
-    <row r="369" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>820</v>
       </c>
@@ -31411,7 +31439,7 @@
         <v/>
       </c>
     </row>
-    <row r="370" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>821</v>
       </c>
@@ -31479,7 +31507,7 @@
         <v/>
       </c>
     </row>
-    <row r="371" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>822</v>
       </c>
@@ -31547,7 +31575,7 @@
         <v/>
       </c>
     </row>
-    <row r="372" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>823</v>
       </c>
@@ -31615,7 +31643,7 @@
         <v/>
       </c>
     </row>
-    <row r="373" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>824</v>
       </c>
@@ -31683,7 +31711,7 @@
         <v/>
       </c>
     </row>
-    <row r="374" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>825</v>
       </c>
@@ -31751,7 +31779,7 @@
         <v/>
       </c>
     </row>
-    <row r="375" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>826</v>
       </c>
@@ -31819,7 +31847,7 @@
         <v/>
       </c>
     </row>
-    <row r="376" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>827</v>
       </c>
@@ -31887,7 +31915,7 @@
         <v/>
       </c>
     </row>
-    <row r="377" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>828</v>
       </c>
@@ -31955,7 +31983,7 @@
         <v/>
       </c>
     </row>
-    <row r="378" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>829</v>
       </c>
@@ -32023,7 +32051,7 @@
         <v/>
       </c>
     </row>
-    <row r="379" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>830</v>
       </c>
@@ -32091,7 +32119,7 @@
         <v/>
       </c>
     </row>
-    <row r="380" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>831</v>
       </c>
@@ -32159,7 +32187,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="381" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>832</v>
       </c>
@@ -32227,7 +32255,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="382" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>833</v>
       </c>
@@ -32295,7 +32323,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="383" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>834</v>
       </c>
@@ -32363,7 +32391,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="384" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>835</v>
       </c>
@@ -32431,7 +32459,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="385" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>836</v>
       </c>
@@ -32499,7 +32527,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="386" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>837</v>
       </c>
@@ -32567,7 +32595,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="387" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>838</v>
       </c>
@@ -32635,7 +32663,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="388" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>839</v>
       </c>
@@ -32703,7 +32731,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="389" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>840</v>
       </c>
@@ -32771,7 +32799,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="390" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>841</v>
       </c>
@@ -32839,7 +32867,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="391" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>842</v>
       </c>
@@ -32907,7 +32935,7 @@
         <v>same</v>
       </c>
     </row>
-    <row r="392" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>843</v>
       </c>
@@ -32975,7 +33003,7 @@
         <v/>
       </c>
     </row>
-    <row r="393" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>844</v>
       </c>
@@ -33043,7 +33071,7 @@
         <v/>
       </c>
     </row>
-    <row r="394" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>845</v>
       </c>
@@ -33111,7 +33139,7 @@
         <v/>
       </c>
     </row>
-    <row r="395" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
         <v>846</v>
       </c>
@@ -33179,7 +33207,7 @@
         <v/>
       </c>
     </row>
-    <row r="396" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>847</v>
       </c>
@@ -33247,7 +33275,7 @@
         <v/>
       </c>
     </row>
-    <row r="397" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>848</v>
       </c>
@@ -33315,7 +33343,7 @@
         <v/>
       </c>
     </row>
-    <row r="398" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>849</v>
       </c>
@@ -33383,7 +33411,7 @@
         <v/>
       </c>
     </row>
-    <row r="399" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>850</v>
       </c>
@@ -33451,7 +33479,7 @@
         <v/>
       </c>
     </row>
-    <row r="400" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>851</v>
       </c>
@@ -33519,7 +33547,7 @@
         <v/>
       </c>
     </row>
-    <row r="401" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>852</v>
       </c>
@@ -33587,7 +33615,7 @@
         <v/>
       </c>
     </row>
-    <row r="402" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>853</v>
       </c>
@@ -33655,7 +33683,7 @@
         <v/>
       </c>
     </row>
-    <row r="403" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>854</v>
       </c>
@@ -33723,7 +33751,7 @@
         <v/>
       </c>
     </row>
-    <row r="404" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>855</v>
       </c>
@@ -33791,7 +33819,7 @@
         <v/>
       </c>
     </row>
-    <row r="405" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>856</v>
       </c>
@@ -33859,7 +33887,7 @@
         <v/>
       </c>
     </row>
-    <row r="406" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>857</v>
       </c>
@@ -33927,7 +33955,7 @@
         <v/>
       </c>
     </row>
-    <row r="407" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>858</v>
       </c>
@@ -33995,7 +34023,7 @@
         <v/>
       </c>
     </row>
-    <row r="408" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
         <v>859</v>
       </c>
@@ -34063,7 +34091,7 @@
         <v/>
       </c>
     </row>
-    <row r="409" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
         <v>860</v>
       </c>
@@ -34131,7 +34159,7 @@
         <v/>
       </c>
     </row>
-    <row r="410" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
         <v>861</v>
       </c>
@@ -34199,7 +34227,7 @@
         <v/>
       </c>
     </row>
-    <row r="411" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A411" t="s">
         <v>862</v>
       </c>
@@ -34267,7 +34295,7 @@
         <v/>
       </c>
     </row>
-    <row r="412" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
         <v>863</v>
       </c>
@@ -34335,7 +34363,7 @@
         <v/>
       </c>
     </row>
-    <row r="413" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
         <v>864</v>
       </c>
@@ -34403,7 +34431,7 @@
         <v/>
       </c>
     </row>
-    <row r="414" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
         <v>865</v>
       </c>
@@ -34471,7 +34499,7 @@
         <v/>
       </c>
     </row>
-    <row r="415" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
         <v>866</v>
       </c>
@@ -34539,7 +34567,7 @@
         <v/>
       </c>
     </row>
-    <row r="416" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
         <v>867</v>
       </c>
@@ -34607,7 +34635,7 @@
         <v/>
       </c>
     </row>
-    <row r="417" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>868</v>
       </c>
@@ -34675,7 +34703,7 @@
         <v/>
       </c>
     </row>
-    <row r="418" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>869</v>
       </c>
@@ -34743,7 +34771,7 @@
         <v/>
       </c>
     </row>
-    <row r="419" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
         <v>870</v>
       </c>
@@ -34811,7 +34839,7 @@
         <v/>
       </c>
     </row>
-    <row r="420" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
         <v>871</v>
       </c>
@@ -34879,7 +34907,7 @@
         <v/>
       </c>
     </row>
-    <row r="421" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
         <v>872</v>
       </c>
@@ -34947,7 +34975,7 @@
         <v/>
       </c>
     </row>
-    <row r="422" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
         <v>873</v>
       </c>
@@ -35015,7 +35043,7 @@
         <v/>
       </c>
     </row>
-    <row r="423" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
         <v>874</v>
       </c>
@@ -35083,7 +35111,7 @@
         <v/>
       </c>
     </row>
-    <row r="424" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
         <v>875</v>
       </c>
@@ -35151,7 +35179,7 @@
         <v/>
       </c>
     </row>
-    <row r="425" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
         <v>876</v>
       </c>
@@ -35219,7 +35247,7 @@
         <v/>
       </c>
     </row>
-    <row r="426" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
         <v>877</v>
       </c>
@@ -35287,7 +35315,7 @@
         <v/>
       </c>
     </row>
-    <row r="427" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>878</v>
       </c>
@@ -35355,7 +35383,7 @@
         <v/>
       </c>
     </row>
-    <row r="428" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>879</v>
       </c>
@@ -35423,7 +35451,7 @@
         <v/>
       </c>
     </row>
-    <row r="429" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>880</v>
       </c>
@@ -35491,7 +35519,7 @@
         <v/>
       </c>
     </row>
-    <row r="430" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
         <v>881</v>
       </c>
@@ -35559,7 +35587,7 @@
         <v/>
       </c>
     </row>
-    <row r="431" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
         <v>882</v>
       </c>
@@ -35627,7 +35655,7 @@
         <v/>
       </c>
     </row>
-    <row r="432" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
         <v>883</v>
       </c>
@@ -35695,7 +35723,7 @@
         <v/>
       </c>
     </row>
-    <row r="433" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
         <v>884</v>
       </c>

</xml_diff>